<commit_message>
Update Templates and Schedule
</commit_message>
<xml_diff>
--- a/Practicas Preprofesionales/horario_practicas.xlsx
+++ b/Practicas Preprofesionales/horario_practicas.xlsx
@@ -112,7 +112,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -137,6 +137,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="1"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="15">
     <border>
@@ -346,7 +352,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -427,6 +433,12 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -709,7 +721,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="C1:Q47"/>
+  <dimension ref="C1:Q46"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="4" width="11.6640625" bestFit="1" customWidth="1"/>
@@ -1690,7 +1702,7 @@
       <c r="F40" s="6">
         <v>9</v>
       </c>
-      <c r="G40" s="6">
+      <c r="G40" s="28">
         <v>10</v>
       </c>
     </row>
@@ -1707,7 +1719,7 @@
       <c r="F41" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="G41" s="4" t="s">
+      <c r="G41" s="29" t="s">
         <v>6</v>
       </c>
       <c r="I41">
@@ -1792,24 +1804,7 @@
       </c>
     </row>
     <row r="46" spans="3:11" x14ac:dyDescent="0.3">
-      <c r="C46" s="6">
-        <v>27</v>
-      </c>
-      <c r="D46" s="6">
-        <v>28</v>
-      </c>
-      <c r="E46" s="6">
-        <v>29</v>
-      </c>
-      <c r="F46" s="6">
-        <v>30</v>
-      </c>
-      <c r="G46" s="6">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="47" spans="3:11" x14ac:dyDescent="0.3">
-      <c r="I47">
+      <c r="I46">
         <f>SUM(I29:I45)</f>
         <v>264</v>
       </c>

</xml_diff>